<commit_message>
PCB Excel report: close the audit's last three Low notes
- the 'priced from a range' caveat appears once, under To verify (was in the range tile,
  the narrative and To verify);
- the volume scatter chart has an inner plot inset so its axis labels clear the border;
- the Summary donut is about 25% smaller, centred beside the composition table.
LibreOffice recalc: 181 formulas, 0 errors, every result equal to the analysis figure.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142L4rKS2AV8rxQTDWMs7dy
</commit_message>
<xml_diff>
--- a/docs/pcb/screens/camera-report-2026-10-06.xlsx
+++ b/docs/pcb/screens/camera-report-2026-10-06.xlsx
@@ -12,7 +12,7 @@
     <sheet sheetId="6" name="Volume &amp; Notes" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Summary'!$A1:$N48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Summary'!$A1:$N47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Cost Breakdown'!$A1:$I27</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Bill of Materials'!$A1:$M28</definedName>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="234">
   <si>
     <t>PCB should-cost report</t>
   </si>
@@ -67,7 +67,7 @@
     <t>China factory gate, packed</t>
   </si>
   <si>
-    <t>Low confidence · 1 line to verify</t>
+    <t>Low confidence · see To verify</t>
   </si>
   <si>
     <t>PPAP · FMEA · DV/PV · audit — not in unit cost</t>
@@ -209,9 +209,6 @@
   </si>
   <si>
     <t>•  China (Shenzhen / Suzhou) is the lowest delivered cost of the 14 countries compared.</t>
-  </si>
-  <si>
-    <t>•  1 line of £1.00+ (£4.64) is priced from a range, not a quote: Image sensor.</t>
   </si>
   <si>
     <t>Not in this unit cost</t>
@@ -2077,7 +2074,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.1"/>
+          <c:y val="0.13"/>
+          <c:w val="0.86"/>
+          <c:h val="0.62"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -2841,15 +2848,15 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3595,7 +3602,7 @@
     <tabColor rgb="FF16325C"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:P48"/>
+  <dimension ref="B1:P47"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -4208,37 +4215,37 @@
       <c r="L42" s="40"/>
       <c r="M42" s="40"/>
     </row>
-    <row r="43" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B43" s="40" t="s">
+    <row r="44" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B44" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="C43" s="40"/>
-      <c r="D43" s="40"/>
-      <c r="E43" s="40"/>
-      <c r="F43" s="40"/>
-      <c r="G43" s="40"/>
-      <c r="H43" s="40"/>
-      <c r="I43" s="40"/>
-      <c r="J43" s="40"/>
-      <c r="K43" s="40"/>
-      <c r="L43" s="40"/>
-      <c r="M43" s="40"/>
-    </row>
-    <row r="45" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B45" s="15" t="s">
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
+      <c r="I44" s="15"/>
+      <c r="J44" s="15"/>
+      <c r="K44" s="15"/>
+      <c r="L44" s="15"/>
+      <c r="M44" s="15"/>
+    </row>
+    <row r="45" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B45" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15"/>
-      <c r="F45" s="15"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="15"/>
-      <c r="I45" s="15"/>
-      <c r="J45" s="15"/>
-      <c r="K45" s="15"/>
-      <c r="L45" s="15"/>
-      <c r="M45" s="15"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="41"/>
+      <c r="F45" s="41"/>
+      <c r="G45" s="41"/>
+      <c r="H45" s="41"/>
+      <c r="I45" s="41"/>
+      <c r="J45" s="41"/>
+      <c r="K45" s="41"/>
+      <c r="L45" s="41"/>
+      <c r="M45" s="41"/>
     </row>
     <row r="46" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46" s="41" t="s">
@@ -4272,24 +4279,8 @@
       <c r="L47" s="41"/>
       <c r="M47" s="41"/>
     </row>
-    <row r="48" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B48" s="41" t="s">
-        <v>64</v>
-      </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="41"/>
-      <c r="I48" s="41"/>
-      <c r="J48" s="41"/>
-      <c r="K48" s="41"/>
-      <c r="L48" s="41"/>
-      <c r="M48" s="41"/>
-    </row>
   </sheetData>
-  <mergeCells count="61">
+  <mergeCells count="60">
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="B3:M3"/>
     <mergeCell ref="B4:M4"/>
@@ -4346,11 +4337,10 @@
     <mergeCell ref="B40:M40"/>
     <mergeCell ref="B41:M41"/>
     <mergeCell ref="B42:M42"/>
-    <mergeCell ref="B43:M43"/>
+    <mergeCell ref="B44:M44"/>
     <mergeCell ref="B45:M45"/>
     <mergeCell ref="B46:M46"/>
     <mergeCell ref="B47:M47"/>
-    <mergeCell ref="B48:M48"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.55" bottom="0.55" header="0.25" footer="0.25"/>
@@ -4402,7 +4392,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -4435,12 +4425,12 @@
     <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
       <c r="E7" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
@@ -4451,22 +4441,22 @@
         <v>31</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D8" s="18" t="s">
         <v>18</v>
       </c>
       <c r="E8" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="G8" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="H8" s="17" t="s">
         <v>71</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4474,7 +4464,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D9" s="21">
         <v>12.7</v>
@@ -4492,7 +4482,7 @@
         <v>3175000</v>
       </c>
       <c r="H9" s="44" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4500,7 +4490,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D10" s="36">
         <v>0.64</v>
@@ -4518,7 +4508,7 @@
         <v>160000</v>
       </c>
       <c r="H10" s="47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4544,7 +4534,7 @@
         <v>67500</v>
       </c>
       <c r="H11" s="44" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4552,7 +4542,7 @@
         <v>4</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D12" s="36">
         <v>0.14</v>
@@ -4570,7 +4560,7 @@
         <v>35000</v>
       </c>
       <c r="H12" s="47" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4578,7 +4568,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D13" s="21">
         <v>0.26</v>
@@ -4596,7 +4586,7 @@
         <v>65000</v>
       </c>
       <c r="H13" s="44" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4604,7 +4594,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D14" s="36">
         <v>0.39</v>
@@ -4622,7 +4612,7 @@
         <v>97500</v>
       </c>
       <c r="H14" s="47" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4630,7 +4620,7 @@
         <v>7</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D15" s="21">
         <v>0.18</v>
@@ -4648,7 +4638,7 @@
         <v>45000</v>
       </c>
       <c r="H15" s="44" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4656,7 +4646,7 @@
         <v>8</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D16" s="36">
         <v>0.13</v>
@@ -4674,7 +4664,7 @@
         <v>32500</v>
       </c>
       <c r="H16" s="47" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4682,7 +4672,7 @@
         <v>9</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D17" s="21">
         <v>0.01</v>
@@ -4700,7 +4690,7 @@
         <v>2500</v>
       </c>
       <c r="H17" s="44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4708,7 +4698,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="49" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" s="50">
         <f>SUM(D9:D17)</f>
@@ -4724,7 +4714,7 @@
         <v>3680000</v>
       </c>
       <c r="H18" s="54" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4732,7 +4722,7 @@
         <v>10</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D19" s="55">
         <v>0</v>
@@ -4750,7 +4740,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4758,7 +4748,7 @@
         <v>11</v>
       </c>
       <c r="C20" s="35" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D20" s="36">
         <v>0.54</v>
@@ -4776,7 +4766,7 @@
         <v>135000</v>
       </c>
       <c r="H20" s="47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -4784,7 +4774,7 @@
         <v>16</v>
       </c>
       <c r="C21" s="57" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D21" s="58">
         <f>D18+SUM(D19:D20)</f>
@@ -4800,7 +4790,7 @@
         <v>3815000</v>
       </c>
       <c r="H21" s="62" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" ht="17.5" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
@@ -4816,7 +4806,7 @@
     </row>
     <row r="24" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
@@ -4828,7 +4818,7 @@
     <row r="25" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="64"/>
       <c r="C25" s="20" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D25" s="65">
         <v>250000</v>
@@ -4837,12 +4827,12 @@
       <c r="F25" s="64"/>
       <c r="G25" s="64"/>
       <c r="H25" s="44" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="66" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C27" s="66"/>
       <c r="D27" s="66"/>
@@ -4871,7 +4861,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{19E32EC8-B523-41E3-830D-51A80AF0AA89}</x14:id>
+          <x14:id>{2EFE3B88-C02E-4D0D-97BA-71E7704815E3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4887,7 +4877,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{19E32EC8-B523-41E3-830D-51A80AF0AA89}">
+          <x14:cfRule type="dataBar" id="{2EFE3B88-C02E-4D0D-97BA-71E7704815E3}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -4949,7 +4939,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -4994,14 +4984,14 @@
     <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" ht="22" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
       <c r="F7" s="15"/>
       <c r="G7" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -5014,34 +5004,34 @@
         <v>31</v>
       </c>
       <c r="C8" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="E8" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="F8" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="G8" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="H8" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="I8" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="I8" s="18" t="s">
+      <c r="J8" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="J8" s="18" t="s">
+      <c r="K8" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="K8" s="17" t="s">
+      <c r="L8" s="17" t="s">
         <v>113</v>
-      </c>
-      <c r="L8" s="17" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
@@ -5049,16 +5039,16 @@
         <v>1</v>
       </c>
       <c r="C9" s="67" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="E9" s="67" t="s">
+        <v>114</v>
+      </c>
+      <c r="F9" s="20" t="s">
         <v>116</v>
-      </c>
-      <c r="E9" s="67" t="s">
-        <v>115</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>117</v>
       </c>
       <c r="G9" s="68">
         <v>49</v>
@@ -5075,7 +5065,7 @@
         <v>0.07165458898731669</v>
       </c>
       <c r="K9" s="71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L9" s="64"/>
     </row>
@@ -5084,16 +5074,16 @@
         <v>2</v>
       </c>
       <c r="C10" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F10" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G10" s="73">
         <v>7</v>
@@ -5110,7 +5100,7 @@
         <v>0.023991491848431933</v>
       </c>
       <c r="K10" s="71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L10" s="76"/>
     </row>
@@ -5119,16 +5109,16 @@
         <v>3</v>
       </c>
       <c r="C11" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E11" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F11" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G11" s="68">
         <v>1</v>
@@ -5145,7 +5135,7 @@
         <v>0.019193193478745544</v>
       </c>
       <c r="K11" s="71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L11" s="64"/>
     </row>
@@ -5154,16 +5144,16 @@
         <v>4</v>
       </c>
       <c r="C12" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E12" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F12" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G12" s="73">
         <v>1</v>
@@ -5180,7 +5170,7 @@
         <v>0.019193193478745544</v>
       </c>
       <c r="K12" s="71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L12" s="76"/>
     </row>
@@ -5189,16 +5179,16 @@
         <v>5</v>
       </c>
       <c r="C13" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>35</v>
       </c>
       <c r="E13" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="F13" s="20" t="s">
         <v>121</v>
-      </c>
-      <c r="F13" s="20" t="s">
-        <v>122</v>
       </c>
       <c r="G13" s="68">
         <v>1</v>
@@ -5215,7 +5205,7 @@
         <v>0.14758402561308126</v>
       </c>
       <c r="K13" s="77" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L13" s="64"/>
     </row>
@@ -5224,16 +5214,16 @@
         <v>6</v>
       </c>
       <c r="C14" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D14" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="E14" s="35" t="s">
         <v>124</v>
       </c>
-      <c r="E14" s="35" t="s">
+      <c r="F14" s="35" t="s">
         <v>125</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>126</v>
       </c>
       <c r="G14" s="73">
         <v>1</v>
@@ -5250,7 +5240,7 @@
         <v>0.10341613917696373</v>
       </c>
       <c r="K14" s="77" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L14" s="76"/>
     </row>
@@ -5259,16 +5249,16 @@
         <v>7</v>
       </c>
       <c r="C15" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D15" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="E15" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="F15" s="20" t="s">
         <v>128</v>
-      </c>
-      <c r="F15" s="20" t="s">
-        <v>129</v>
       </c>
       <c r="G15" s="68">
         <v>1</v>
@@ -5285,7 +5275,7 @@
         <v>0.06441352053851725</v>
       </c>
       <c r="K15" s="77" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L15" s="64"/>
     </row>
@@ -5294,16 +5284,16 @@
         <v>8</v>
       </c>
       <c r="C16" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D16" s="35" t="s">
+        <v>129</v>
+      </c>
+      <c r="E16" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="E16" s="35" t="s">
+      <c r="F16" s="35" t="s">
         <v>131</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>132</v>
       </c>
       <c r="G16" s="73">
         <v>1</v>
@@ -5320,7 +5310,7 @@
         <v>0.013210899407448231</v>
       </c>
       <c r="K16" s="77" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L16" s="76"/>
     </row>
@@ -5329,16 +5319,16 @@
         <v>9</v>
       </c>
       <c r="C17" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D17" s="20" t="s">
         <v>34</v>
       </c>
       <c r="E17" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="F17" s="20" t="s">
         <v>133</v>
-      </c>
-      <c r="F17" s="20" t="s">
-        <v>134</v>
       </c>
       <c r="G17" s="68">
         <v>1</v>
@@ -5355,7 +5345,7 @@
         <v>0.1651777863019314</v>
       </c>
       <c r="K17" s="77" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L17" s="64"/>
     </row>
@@ -5364,16 +5354,16 @@
         <v>10</v>
       </c>
       <c r="C18" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E18" s="72" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G18" s="73">
         <v>16</v>
@@ -5390,7 +5380,7 @@
         <v>0.006580523478427043</v>
       </c>
       <c r="K18" s="71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L18" s="76"/>
     </row>
@@ -5399,16 +5389,16 @@
         <v>11</v>
       </c>
       <c r="C19" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E19" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F19" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G19" s="68">
         <v>1</v>
@@ -5425,17 +5415,17 @@
         <v>0.36558463769039135</v>
       </c>
       <c r="K19" s="71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L19" s="78" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="79"/>
       <c r="C20" s="79"/>
       <c r="D20" s="57" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E20" s="79"/>
       <c r="F20" s="79"/>
@@ -5457,7 +5447,7 @@
     </row>
     <row r="22" ht="22" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
@@ -5474,7 +5464,7 @@
       <c r="B23" s="64"/>
       <c r="C23" s="64"/>
       <c r="D23" s="20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E23" s="20"/>
       <c r="F23" s="20"/>
@@ -5492,7 +5482,7 @@
       <c r="B24" s="64"/>
       <c r="C24" s="64"/>
       <c r="D24" s="20" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E24" s="20"/>
       <c r="F24" s="20"/>
@@ -5510,7 +5500,7 @@
       <c r="B25" s="64"/>
       <c r="C25" s="64"/>
       <c r="D25" s="20" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E25" s="20"/>
       <c r="F25" s="20"/>
@@ -5540,7 +5530,7 @@
     </row>
     <row r="27" ht="30" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="66" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C27" s="66"/>
       <c r="D27" s="66"/>
@@ -5555,7 +5545,7 @@
     </row>
     <row r="28" ht="30" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="66" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C28" s="66"/>
       <c r="D28" s="66"/>
@@ -5635,7 +5625,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -5680,14 +5670,14 @@
     <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" ht="22" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
       <c r="F7" s="15"/>
       <c r="H7" s="15" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I7" s="15"/>
       <c r="J7" s="16" t="s">
@@ -5701,13 +5691,13 @@
         <v>48</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D8" s="20"/>
       <c r="E8" s="20"/>
       <c r="F8" s="20"/>
       <c r="H8" s="20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I8" s="20"/>
       <c r="J8" s="20"/>
@@ -5738,16 +5728,16 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>150</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>151</v>
       </c>
       <c r="D10" s="20"/>
       <c r="E10" s="20"/>
       <c r="F10" s="20"/>
       <c r="H10" s="20" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I10" s="20"/>
       <c r="J10" s="20"/>
@@ -5758,16 +5748,16 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="47" t="s">
+        <v>152</v>
+      </c>
+      <c r="C11" s="35" t="s">
         <v>153</v>
-      </c>
-      <c r="C11" s="35" t="s">
-        <v>154</v>
       </c>
       <c r="D11" s="35"/>
       <c r="E11" s="35"/>
       <c r="F11" s="35"/>
       <c r="H11" s="35" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I11" s="35"/>
       <c r="J11" s="35"/>
@@ -5778,16 +5768,16 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="44" t="s">
+        <v>155</v>
+      </c>
+      <c r="C12" s="20" t="s">
         <v>156</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>157</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="20"/>
       <c r="F12" s="20"/>
       <c r="H12" s="20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I12" s="20"/>
       <c r="J12" s="20"/>
@@ -5798,16 +5788,16 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="47" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C13" s="35" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D13" s="35"/>
       <c r="E13" s="35"/>
       <c r="F13" s="35"/>
       <c r="H13" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="20"/>
@@ -5819,16 +5809,16 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="44" t="s">
+        <v>160</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>161</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>162</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
       <c r="F14" s="20"/>
       <c r="H14" s="20" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I14" s="20"/>
       <c r="J14" s="20"/>
@@ -5840,16 +5830,16 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="47" t="s">
+        <v>163</v>
+      </c>
+      <c r="C15" s="35" t="s">
         <v>164</v>
-      </c>
-      <c r="C15" s="35" t="s">
-        <v>165</v>
       </c>
       <c r="D15" s="35"/>
       <c r="E15" s="35"/>
       <c r="F15" s="35"/>
       <c r="H15" s="20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I15" s="20"/>
       <c r="J15" s="20"/>
@@ -5861,7 +5851,7 @@
     </row>
     <row r="16" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H16" s="84" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I16" s="84"/>
       <c r="J16" s="84"/>
@@ -5884,7 +5874,7 @@
     </row>
     <row r="19" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H19" s="20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I19" s="20"/>
       <c r="J19" s="20"/>
@@ -5896,7 +5886,7 @@
     </row>
     <row r="20" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H20" s="35" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I20" s="35"/>
       <c r="J20" s="35"/>
@@ -5908,7 +5898,7 @@
     </row>
     <row r="21" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H21" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I21" s="20"/>
       <c r="J21" s="20"/>
@@ -5920,7 +5910,7 @@
     </row>
     <row r="22" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H22" s="84" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I22" s="84"/>
       <c r="J22" s="84"/>
@@ -5932,14 +5922,14 @@
     </row>
     <row r="24" ht="22" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
       <c r="E24" s="15"/>
       <c r="F24" s="15"/>
       <c r="G24" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H24" s="16"/>
       <c r="I24" s="16"/>
@@ -5959,10 +5949,10 @@
     <row r="34" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="15" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="86" t="s">
+        <v>171</v>
+      </c>
+      <c r="H35" s="86" t="s">
         <v>172</v>
-      </c>
-      <c r="H35" s="86" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5978,7 +5968,7 @@
     <row r="46" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="47" ht="15" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="86" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6084,7 +6074,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -6135,7 +6125,7 @@
     <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" ht="22" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
@@ -6144,7 +6134,7 @@
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
       <c r="I7" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J7" s="16"/>
       <c r="K7" s="16"/>
@@ -6154,43 +6144,43 @@
     </row>
     <row r="8" ht="30" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="C8" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="D8" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>180</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>181</v>
       </c>
       <c r="F8" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G8" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="H8" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="I8" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="I8" s="18" t="s">
+      <c r="J8" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="J8" s="18" t="s">
+      <c r="K8" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="L8" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="L8" s="18" t="s">
+      <c r="M8" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="M8" s="17" t="s">
+      <c r="N8" s="87" t="s">
         <v>188</v>
-      </c>
-      <c r="N8" s="87" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
@@ -6198,7 +6188,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="89" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D9" s="90">
         <v>13.34</v>
@@ -6244,7 +6234,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D10" s="36">
         <v>13.95</v>
@@ -6290,7 +6280,7 @@
         <v>3</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D11" s="21">
         <v>13.8</v>
@@ -6336,7 +6326,7 @@
         <v>4</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D12" s="36">
         <v>14.1</v>
@@ -6382,7 +6372,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D13" s="21">
         <v>14.4</v>
@@ -6428,7 +6418,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D14" s="36">
         <v>13.65</v>
@@ -6474,7 +6464,7 @@
         <v>7</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D15" s="21">
         <v>14.86</v>
@@ -6520,7 +6510,7 @@
         <v>8</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D16" s="36">
         <v>13.95</v>
@@ -6566,7 +6556,7 @@
         <v>9</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D17" s="21">
         <v>15.92</v>
@@ -6612,7 +6602,7 @@
         <v>10</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D18" s="36">
         <v>16.07</v>
@@ -6658,7 +6648,7 @@
         <v>11</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D19" s="21">
         <v>17.89</v>
@@ -6704,7 +6694,7 @@
         <v>12</v>
       </c>
       <c r="C20" s="35" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D20" s="36">
         <v>17.44</v>
@@ -6750,7 +6740,7 @@
         <v>13</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D21" s="21">
         <v>18.5</v>
@@ -6796,7 +6786,7 @@
         <v>14</v>
       </c>
       <c r="C22" s="35" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D22" s="36">
         <v>18.19</v>
@@ -6839,7 +6829,7 @@
     </row>
     <row r="23" ht="30" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" s="66" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C23" s="66"/>
       <c r="D23" s="66"/>
@@ -6915,7 +6905,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -6963,7 +6953,7 @@
     <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
@@ -6971,7 +6961,7 @@
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
       <c r="H7" s="16" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="16"/>
@@ -6981,13 +6971,13 @@
     </row>
     <row r="8" ht="42" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>208</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="D8" s="18" t="s">
         <v>209</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.25">
@@ -7102,14 +7092,14 @@
     </row>
     <row r="19" ht="17.5" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="66" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C19" s="66"/>
       <c r="D19" s="66"/>
     </row>
     <row r="26" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" s="15" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
@@ -7117,7 +7107,7 @@
       <c r="F26" s="15"/>
       <c r="G26" s="15"/>
       <c r="H26" s="16" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="I26" s="16"/>
       <c r="J26" s="16"/>
@@ -7127,19 +7117,19 @@
     </row>
     <row r="27" ht="30" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B27" s="17" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G27" s="18"/>
       <c r="H27" s="18"/>
       <c r="I27" s="18"/>
       <c r="J27" s="18" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K27" s="18"/>
       <c r="L27" s="18"/>
@@ -7147,7 +7137,7 @@
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B28" s="20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C28" s="20"/>
       <c r="D28" s="20"/>
@@ -7168,7 +7158,7 @@
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B29" s="35" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C29" s="35"/>
       <c r="D29" s="35"/>
@@ -7189,7 +7179,7 @@
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B30" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C30" s="20"/>
       <c r="D30" s="20"/>
@@ -7210,7 +7200,7 @@
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B31" s="35" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C31" s="35"/>
       <c r="D31" s="35"/>
@@ -7231,7 +7221,7 @@
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B32" s="29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C32" s="29"/>
       <c r="D32" s="29"/>
@@ -7253,7 +7243,7 @@
     </row>
     <row r="34" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B34" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C34" s="15"/>
       <c r="D34" s="15"/>
@@ -7269,7 +7259,7 @@
     </row>
     <row r="35" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35" s="113" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C35" s="113"/>
       <c r="D35" s="113"/>
@@ -7285,7 +7275,7 @@
     </row>
     <row r="36" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B36" s="113" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C36" s="113"/>
       <c r="D36" s="113"/>
@@ -7301,7 +7291,7 @@
     </row>
     <row r="38" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B38" s="15" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C38" s="15"/>
       <c r="D38" s="15"/>
@@ -7317,7 +7307,7 @@
     </row>
     <row r="39" ht="30" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B39" s="113" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C39" s="113"/>
       <c r="D39" s="113"/>
@@ -7333,7 +7323,7 @@
     </row>
     <row r="41" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B41" s="15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C41" s="15"/>
       <c r="D41" s="15"/>
@@ -7349,7 +7339,7 @@
     </row>
     <row r="42" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B42" s="113" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C42" s="113"/>
       <c r="D42" s="113"/>
@@ -7365,7 +7355,7 @@
     </row>
     <row r="44" ht="22" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B44" s="15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C44" s="15"/>
       <c r="D44" s="15"/>
@@ -7381,7 +7371,7 @@
     </row>
     <row r="45" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B45" s="113" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C45" s="113"/>
       <c r="D45" s="113"/>
@@ -7397,7 +7387,7 @@
     </row>
     <row r="46" ht="30" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46" s="113" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C46" s="113"/>
       <c r="D46" s="113"/>
@@ -7413,7 +7403,7 @@
     </row>
     <row r="47" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B47" s="113" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C47" s="113"/>
       <c r="D47" s="113"/>
@@ -7429,7 +7419,7 @@
     </row>
     <row r="48" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B48" s="113" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C48" s="113"/>
       <c r="D48" s="113"/>
@@ -7445,7 +7435,7 @@
     </row>
     <row r="49" ht="17.5" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="113" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C49" s="113"/>
       <c r="D49" s="113"/>

</xml_diff>